<commit_message>
Cambiar el acento ocre por azul petróleo en todo el sitio
El ocre se parecía demasiado a una paleta reconocible y le restaba
identidad propia al sitio. El acento pasa a azul petróleo (#0E5A66, con
#7FC4CC sobre fondo oscuro) en figuras, ilustración del inicio, títulos,
botones, enlaces, favicon, imagen para redes y el test en Excel, donde el
estado "Débil" pasa a un rosado suave. Los tokens de Tailwind se
renombran de `ocre` a `acento` para que el nombre no ate el código a un
color.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/descargas/test-de-madurez-operativa.xlsx
+++ b/public/descargas/test-de-madurez-operativa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jrive\Procesos-Claros-WS\Procesos-Claros-WS\public\descargas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752A5FD5-2BEF-464B-BB41-FAEA80EAEB83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984192DE-7943-48F4-AD47-47F5AADA7BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -366,7 +366,7 @@
     <font>
       <b/>
       <sz val="13"/>
-      <color rgb="FFB45309"/>
+      <color rgb="FF0E5A66"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -389,13 +389,13 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFB45309"/>
+      <color rgb="FF0E5A66"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
-      <color rgb="FFB45309"/>
+      <color rgb="FF0E5A66"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -424,7 +424,7 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FFB45309"/>
+      <color rgb="FF0E5A66"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -615,8 +615,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7C4"/>
-          <bgColor rgb="FFF8D7C4"/>
+          <fgColor rgb="FFF2D5D5"/>
+          <bgColor rgb="FFF2D5D5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -668,11 +668,11 @@
           <c:order val="0"/>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="B45309"/>
+              <a:srgbClr val="0E5A66"/>
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="B45309"/>
+                <a:srgbClr val="0E5A66"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -755,7 +755,7 @@
                   </a:solidFill>
                   <a:ln>
                     <a:solidFill>
-                      <a:srgbClr val="B45309"/>
+                      <a:srgbClr val="0E5A66"/>
                     </a:solidFill>
                     <a:prstDash val="solid"/>
                   </a:ln>
@@ -763,7 +763,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-07B6-491B-8CC7-35605398AD66}"/>
+              <c16:uniqueId val="{00000000-9A37-4A7D-BEBC-AED4B937FBDE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1321,7 +1321,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
-    <tabColor rgb="FFB45309"/>
+    <tabColor rgb="FF0E5A66"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:G29"/>
@@ -2119,9 +2119,9 @@
     <hyperlink ref="B29" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup scale="54" orientation="landscape" r:id="rId2"/>
-  <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>